<commit_message>
p1: welcome message on /start and /help
</commit_message>
<xml_diff>
--- a/data/satech_dun_field_log_sample.xlsx
+++ b/data/satech_dun_field_log_sample.xlsx
@@ -3869,7 +3869,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="19" min="1" max="1"/>
@@ -4632,6 +4632,249 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="35" t="inlineStr">
+        <is>
+          <t>start_hello</t>
+        </is>
+      </c>
+      <c r="B29" s="35" t="inlineStr">
+        <is>
+          <t>Hi {name}! Today is {date}.</t>
+        </is>
+      </c>
+      <c r="C29" s="35" t="inlineStr">
+        <is>
+          <t>Hola {name}! Avui és {date}.</t>
+        </is>
+      </c>
+      <c r="D29" s="35" t="inlineStr">
+        <is>
+          <t>¡Hola {name}! Hoy es {date}.</t>
+        </is>
+      </c>
+      <c r="E29" s="35" t="inlineStr">
+        <is>
+          <t>Привет, {name}! Сегодня {date}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="35" t="inlineStr">
+        <is>
+          <t>start_parcels</t>
+        </is>
+      </c>
+      <c r="B30" s="35" t="inlineStr">
+        <is>
+          <t>🌱 Your parcels (DUN {campaign}):</t>
+        </is>
+      </c>
+      <c r="C30" s="35" t="inlineStr">
+        <is>
+          <t>🌱 Les teves parcel·les (DUN {campaign}):</t>
+        </is>
+      </c>
+      <c r="D30" s="35" t="inlineStr">
+        <is>
+          <t>🌱 Tus parcelas (DUN {campaign}):</t>
+        </is>
+      </c>
+      <c r="E30" s="35" t="inlineStr">
+        <is>
+          <t>🌱 Ваши участки (DUN {campaign}):</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="35" t="inlineStr">
+        <is>
+          <t>start_today</t>
+        </is>
+      </c>
+      <c r="B31" s="35" t="inlineStr">
+        <is>
+          <t>Logged today: {n} records.</t>
+        </is>
+      </c>
+      <c r="C31" s="35" t="inlineStr">
+        <is>
+          <t>Registrat avui: {n} registres.</t>
+        </is>
+      </c>
+      <c r="D31" s="35" t="inlineStr">
+        <is>
+          <t>Registrado hoy: {n} registros.</t>
+        </is>
+      </c>
+      <c r="E31" s="35" t="inlineStr">
+        <is>
+          <t>Сегодня записано: {n}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="35" t="inlineStr">
+        <is>
+          <t>start_functions</t>
+        </is>
+      </c>
+      <c r="B32" s="35" t="inlineStr">
+        <is>
+          <t>What I can do:</t>
+        </is>
+      </c>
+      <c r="C32" s="35" t="inlineStr">
+        <is>
+          <t>Què puc fer:</t>
+        </is>
+      </c>
+      <c r="D32" s="35" t="inlineStr">
+        <is>
+          <t>Qué puedo hacer:</t>
+        </is>
+      </c>
+      <c r="E32" s="35" t="inlineStr">
+        <is>
+          <t>Что я умею:</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="35" t="inlineStr">
+        <is>
+          <t>func_voice</t>
+        </is>
+      </c>
+      <c r="B33" s="35" t="inlineStr">
+        <is>
+          <t>🎤 Send a voice note about your work — I turn it into a record</t>
+        </is>
+      </c>
+      <c r="C33" s="35" t="inlineStr">
+        <is>
+          <t>🎤 Envia una nota de veu sobre la feina — la converteixo en un registre</t>
+        </is>
+      </c>
+      <c r="D33" s="35" t="inlineStr">
+        <is>
+          <t>🎤 Envía una nota de voz sobre tu trabajo — la convierto en un registro</t>
+        </is>
+      </c>
+      <c r="E33" s="35" t="inlineStr">
+        <is>
+          <t>🎤 Отправьте голосовое о работе — я превращу его в запись</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="35" t="inlineStr">
+        <is>
+          <t>func_confirm</t>
+        </is>
+      </c>
+      <c r="B34" s="35" t="inlineStr">
+        <is>
+          <t>✅ Check the card and confirm, or ✏️ say what to fix</t>
+        </is>
+      </c>
+      <c r="C34" s="35" t="inlineStr">
+        <is>
+          <t>✅ Revisa la fitxa i confirma, o ✏️ digues què cal corregir</t>
+        </is>
+      </c>
+      <c r="D34" s="35" t="inlineStr">
+        <is>
+          <t>✅ Revisa la ficha y confirma, o ✏️ di qué hay que corregir</t>
+        </is>
+      </c>
+      <c r="E34" s="35" t="inlineStr">
+        <is>
+          <t>✅ Проверьте карточку и подтвердите или ✏️ скажите, что исправить</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="35" t="inlineStr">
+        <is>
+          <t>func_report</t>
+        </is>
+      </c>
+      <c r="B35" s="35" t="inlineStr">
+        <is>
+          <t>📊 /report — your field log as Excel</t>
+        </is>
+      </c>
+      <c r="C35" s="35" t="inlineStr">
+        <is>
+          <t>📊 /report — el teu quadern de camp en Excel</t>
+        </is>
+      </c>
+      <c r="D35" s="35" t="inlineStr">
+        <is>
+          <t>📊 /report — tu cuaderno de campo en Excel</t>
+        </is>
+      </c>
+      <c r="E35" s="35" t="inlineStr">
+        <is>
+          <t>📊 /report — журнал работ в Excel</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="35" t="inlineStr">
+        <is>
+          <t>func_help</t>
+        </is>
+      </c>
+      <c r="B36" s="35" t="inlineStr">
+        <is>
+          <t>❓ /help — show this message again</t>
+        </is>
+      </c>
+      <c r="C36" s="35" t="inlineStr">
+        <is>
+          <t>❓ /help — torna a mostrar aquest missatge</t>
+        </is>
+      </c>
+      <c r="D36" s="35" t="inlineStr">
+        <is>
+          <t>❓ /help — vuelve a mostrar este mensaje</t>
+        </is>
+      </c>
+      <c r="E36" s="35" t="inlineStr">
+        <is>
+          <t>❓ /help — показать это сообщение снова</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="35" t="inlineStr">
+        <is>
+          <t>start_example</t>
+        </is>
+      </c>
+      <c r="B37" s="35" t="inlineStr">
+        <is>
+          <t>Try: “Today I watered parcel 2, 120 cubic metres.”</t>
+        </is>
+      </c>
+      <c r="C37" s="35" t="inlineStr">
+        <is>
+          <t>Prova: «Avui he regat la parcel·la 2, 120 metres cúbics.»</t>
+        </is>
+      </c>
+      <c r="D37" s="35" t="inlineStr">
+        <is>
+          <t>Prueba: «Hoy he regado la parcela 2, 120 metros cúbicos.»</t>
+        </is>
+      </c>
+      <c r="E37" s="35" t="inlineStr">
+        <is>
+          <t>Например: «Сегодня полил второй участок, 120 кубометров».</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>